<commit_message>
reached final shape of payroll obj
</commit_message>
<xml_diff>
--- a/Active May.xlsx
+++ b/Active May.xlsx
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Voda!$A$1:$D$17</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>Name</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>sara</t>
+  </si>
+  <si>
+    <t>ahmed</t>
   </si>
 </sst>
 </file>
@@ -194,7 +197,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -217,13 +220,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -255,6 +269,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -742,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="10.33203125" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -1012,6 +1032,20 @@
         <v>1</v>
       </c>
       <c r="E17" s="8"/>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="12">
+        <v>100</v>
+      </c>
+      <c r="C18" s="12">
+        <v>70</v>
+      </c>
+      <c r="D18" s="1">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
working lower standards except for exports
</commit_message>
<xml_diff>
--- a/Active May.xlsx
+++ b/Active May.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23256" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23256" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Voda" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
   <si>
     <t>Name</t>
   </si>
@@ -72,9 +72,6 @@
     <t>Asmaa</t>
   </si>
   <si>
-    <t>Malak</t>
-  </si>
-  <si>
     <t>Aya Ahmed</t>
   </si>
   <si>
@@ -132,7 +129,7 @@
     <t>sara</t>
   </si>
   <si>
-    <t>ahmed</t>
+    <t>Ahmed</t>
   </si>
 </sst>
 </file>
@@ -197,7 +194,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -220,24 +217,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -269,12 +255,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -762,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="10.33203125" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -827,7 +807,7 @@
         <v>40</v>
       </c>
       <c r="C4" s="4">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D4" s="8">
         <v>6</v>
@@ -898,13 +878,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="4" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B9" s="4">
         <v>35</v>
       </c>
       <c r="C9" s="4">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="D9" s="8">
         <v>5</v>
@@ -913,7 +893,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="4">
         <v>35</v>
@@ -928,7 +908,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="4">
         <v>42</v>
@@ -943,7 +923,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" s="4">
         <v>30</v>
@@ -958,7 +938,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="4">
         <v>40</v>
@@ -975,7 +955,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="4">
         <v>30</v>
@@ -990,7 +970,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="8">
         <v>30</v>
@@ -1005,7 +985,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="8">
         <v>30</v>
@@ -1020,7 +1000,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="4">
         <v>35</v>
@@ -1032,20 +1012,6 @@
         <v>1</v>
       </c>
       <c r="E17" s="8"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="12">
-        <v>100</v>
-      </c>
-      <c r="C18" s="12">
-        <v>70</v>
-      </c>
-      <c r="D18" s="1">
-        <v>2</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1078,23 +1044,23 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="C2" s="4">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="4">
         <v>3</v>
@@ -1106,10 +1072,10 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" s="4">
         <v>4</v>
@@ -1121,10 +1087,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="4">
         <v>5</v>
@@ -1134,10 +1100,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="4">
         <v>4</v>
@@ -1149,10 +1115,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" s="4">
         <v>5</v>
@@ -1161,15 +1127,15 @@
         <v>3</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" s="4">
         <v>9</v>
@@ -1181,10 +1147,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4">
         <v>2</v>
@@ -1193,15 +1159,15 @@
         <v>8</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="4">
         <v>2</v>
@@ -1210,7 +1176,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:5">

</xml_diff>